<commit_message>
Implemented excel master agent workflow
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,89 +476,98 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>ai_draft</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>processed_image</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>ai_draft</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cloud Computing Summit 2026</t>
+          <t>AI &amp; Future Meetup</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A deep dive into serverless architectures and hybrid cloud solutions.</t>
+          <t>Exploring the impact of Llama 3 models on local development.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bangalore Tech Hub</t>
+          <t>Online (Zoom)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>March 25, 2026 - 10:00 AM</t>
+          <t>April 2, 2026 - 6:00 PM</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dr. Aris V.</t>
+          <t>Siddharth S.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1Z8B6M9z3hG_g_L3v_y_6_y/view?usp=sharing</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>https://drive.google.com/file/d/16M1mKuGq4-68TluO6ltkZ_NoR-sQK4a-/view?usp=sharing</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Review Required</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://meetup.com/cloud-summit</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Unexpected Response Structure: 'data'</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+          <t>https://meetup.com/ai-future</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>🚀 AI &amp; Future Meetup 🚀
+• Speaker: Siddharth S.
+• Where: Online (Zoom)
+• Topic: Llama 3 models' impact on local development
+• When: Apr 2, 6:00 PM
+Join now! 👉 https://meetup.com/ai-future #AI #FutureMeetup</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://d.uguu.se/VrbkKqfi.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AI &amp; Future Meetup</t>
+          <t>LLM VS VLLM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Exploring the impact of Llama 3 models on local development.</t>
+          <t>HOW TO INTEGRATE THE BOTH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Online (Zoom)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>April 2, 2026 - 6:00 PM</t>
-        </is>
-      </c>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Siddharth S.</t>
+          <t>SIDDD</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/16M1mKuGq4-68TluO6ltkZ_NoR-sQK4a-/view?usp=sharing</t>
+          <t>https://drive.google.com/file/d/1KoN8fuS4sogEXquQ2d8qimNjktMpSH0M/view?usp=sharing</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -566,132 +575,21 @@
           <t>Review Required</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://meetup.com/ai-future</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://d.uguu.se/YokPfxag.jpg</t>
+          <t>🚀 LLM VS VLLM: The Ultimate Showdown! 🤖
+• Speaker: SIDDD
+• Venue: USA
+• Learn how to integrate LLM &amp; VLLM for maximum impact! 💡
+• Time: [Insert Time] ⏰
+Click the link to join: [Insert Link] #LLM #VLLM #AI</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>🚀 AI &amp; Future Meetup 🚀
-• Speaker: Siddharth S.
-• Where: Online (Zoom)
-• Topic: Exploring Llama 3's impact on local development
-• When: Apr 2, 6:00 PM
-Join now: https://meetup.com/ai-future #AI #FutureTech #Meetup</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Retro Gaming Night</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Join us for a nostalgic evening playing classic 8-bit games!</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>The Game Zone, Delhi</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>April 15, 2026 - 7:00 PM</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Team Antigravity</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/12ydKQydCgZBSrq_FKGgWZpyZlA7XQ734/view?usp=sharing</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>https://meetup.com/retro-gaming</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>https://d.uguu.se/tNLHFaRd.jpg</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Get ready for a blast from the past! 🚀 Introducing Retro Gaming Night 🎮
-• Speaker: Team Antigravity
-• Venue: The Game Zone, Delhi 📍
-• Join us for a nostalgic 8-bit gaming night! 🕹️
-• When: Apr 15, 7:00 PM ⏰
-• Register: https://meetup.com/retro-gaming #RetroGaming</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>how ai can be superfriendly</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">join to know how we can do it most efficiently </t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>dubai</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2023-03-01 00:00:00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">abhay </t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1RaHk79nJ-f_NpPXbJ3empfHt-DQ6uU1d/view?usp=sharing</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>https://d.uguu.se/AinxxFPl.jpg</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>🚀 'How AI Can Be Superfriendly' 🤖 with Abhay! 📢 Join us in Dubai 📍 to discover the secrets of efficient AI integration 🤔 When: March 1st, 00:00 🕰️ Don't miss out! #AI #Superfriendly #Dubai</t>
+          <t>https://o.uguu.se/nbAEDioe.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Excel sync cache flow and clean generated files
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,7 +518,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Review Required</t>
+          <t>Posted</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -526,70 +526,19 @@
           <t>https://meetup.com/ai-future</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://twitter.com/ABHAYSHIND59213/status/2034345078915768468</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>🚀 AI &amp; Future Meetup 🚀
-• Speaker: Siddharth S.
-• Where: Online (Zoom)
-• Topic: Llama 3 models' impact on local development
-• When: Apr 2, 6:00 PM
-Join now! 👉 https://meetup.com/ai-future #AI #FutureMeetup</t>
+          <t>🚀 Explore the Future of AI! 🤖 Join Siddharth S. on April 2, 2026 at 6:00 PM on Zoom to discuss Llama 3 models' impact on local development. 📊 Register now: https://meetup.com/ai-future #AI #FutureMeetup #Llama3</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://d.uguu.se/VrbkKqfi.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LLM VS VLLM</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>HOW TO INTEGRATE THE BOTH</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>SIDDD</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1KoN8fuS4sogEXquQ2d8qimNjktMpSH0M/view?usp=sharing</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>🚀 LLM VS VLLM: The Ultimate Showdown! 🤖
-• Speaker: SIDDD
-• Venue: USA
-• Learn how to integrate LLM &amp; VLLM for maximum impact! 💡
-• Time: [Insert Time] ⏰
-Click the link to join: [Insert Link] #LLM #VLLM #AI</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://o.uguu.se/nbAEDioe.jpg</t>
+          <t>https://n.uguu.se/rJxCPucz.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>